<commit_message>
fix: Arrumando a planinha de requisitos.
</commit_message>
<xml_diff>
--- a/requisitos-sistema/requisitos_estoque_cozinha.xlsx
+++ b/requisitos-sistema/requisitos_estoque_cozinha.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://institutogerminare-my.sharepoint.com/personal/davi_souza_institutojef_org_br/Documents/Área de Trabalho/GerminaT 2/inventra/engenharia-e-qualidade-de-software/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://institutogerminare-my.sharepoint.com/personal/davi_souza_institutojef_org_br/Documents/Área de Trabalho/GerminaT 2/inventra/engenharia-e-qualidade-de-software/requisitos-sistema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{61C9EADD-2906-4450-8165-81B34D94D9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D213BA10-9BB8-4C6E-BC87-71910AB1B0CD}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{61C9EADD-2906-4450-8165-81B34D94D9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66F54511-7A6D-46B5-A2FC-6BD16416E2F9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="143">
   <si>
     <t>Código</t>
   </si>
@@ -185,9 +185,6 @@
     <t>Apresentar indicadores e métricas do estoque.</t>
   </si>
   <si>
-    <t>RF20</t>
-  </si>
-  <si>
     <t>Autenticação</t>
   </si>
   <si>
@@ -324,12 +321,6 @@
   </si>
   <si>
     <t>RF23</t>
-  </si>
-  <si>
-    <t>Transferência entre cozinhas</t>
-  </si>
-  <si>
-    <t>Permitir transferir produtos de uma cozinha para outra, com registro de origem, destino, quantidade e motivo.</t>
   </si>
   <si>
     <t>RF24</t>
@@ -585,8 +576,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C92AE2FF-755C-4500-BBA2-265A9C2A3D10}" name="Tabela1" displayName="Tabela1" ref="A1:C30" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:C30" xr:uid="{C92AE2FF-755C-4500-BBA2-265A9C2A3D10}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C92AE2FF-755C-4500-BBA2-265A9C2A3D10}" name="Tabela1" displayName="Tabela1" ref="A1:C29" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:C29" xr:uid="{C92AE2FF-755C-4500-BBA2-265A9C2A3D10}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{C7205364-51EA-4410-8A03-368DA3CA1DA5}" name="Código" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{F6C5F0B6-B179-41B7-BECF-69D1011F0C93}" name="Título"/>
@@ -893,7 +884,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
@@ -991,7 +982,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B9" t="s">
         <v>28</v>
@@ -1013,7 +1004,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B11" t="s">
         <v>34</v>
@@ -1093,10 +1084,10 @@
         <v>45</v>
       </c>
       <c r="B18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" t="s">
         <v>55</v>
-      </c>
-      <c r="C18" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -1104,10 +1095,10 @@
         <v>48</v>
       </c>
       <c r="B19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="s">
         <v>58</v>
-      </c>
-      <c r="C19" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1115,18 +1106,18 @@
         <v>51</v>
       </c>
       <c r="B20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" t="s">
         <v>61</v>
       </c>
-      <c r="C20" t="s">
-        <v>62</v>
-      </c>
       <c r="D20" s="3" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s">
         <v>101</v>
@@ -1137,7 +1128,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B22" t="s">
         <v>104</v>
@@ -1148,7 +1139,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>60</v>
+        <v>99</v>
       </c>
       <c r="B23" t="s">
         <v>107</v>
@@ -1162,10 +1153,10 @@
         <v>100</v>
       </c>
       <c r="B24" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="C24" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1173,10 +1164,10 @@
         <v>103</v>
       </c>
       <c r="B25" t="s">
-        <v>132</v>
+        <v>111</v>
       </c>
       <c r="C25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1184,10 +1175,10 @@
         <v>106</v>
       </c>
       <c r="B26" t="s">
+        <v>113</v>
+      </c>
+      <c r="C26" t="s">
         <v>114</v>
-      </c>
-      <c r="C26" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1195,48 +1186,37 @@
         <v>109</v>
       </c>
       <c r="B27" t="s">
+        <v>115</v>
+      </c>
+      <c r="C27" t="s">
         <v>116</v>
-      </c>
-      <c r="C27" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C28" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B29" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="C29" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>135</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="B30" t="s">
-        <v>136</v>
-      </c>
-      <c r="C30" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -1270,194 +1250,194 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s">
         <v>65</v>
-      </c>
-      <c r="C2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" t="s">
         <v>68</v>
-      </c>
-      <c r="C3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" t="s">
         <v>71</v>
-      </c>
-      <c r="C4" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" t="s">
         <v>74</v>
-      </c>
-      <c r="C5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" t="s">
         <v>77</v>
-      </c>
-      <c r="C6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" t="s">
         <v>80</v>
-      </c>
-      <c r="C7" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" t="s">
         <v>83</v>
-      </c>
-      <c r="C8" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" t="s">
         <v>87</v>
-      </c>
-      <c r="C9" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" t="s">
         <v>90</v>
-      </c>
-      <c r="C10" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" t="s">
         <v>93</v>
-      </c>
-      <c r="C11" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" t="s">
         <v>96</v>
-      </c>
-      <c r="C12" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C14" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B15" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C15" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B16" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C16" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B17" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C17" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B18" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C18" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B19" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
fix: Refinando a planilha e a doc de requisitos.
</commit_message>
<xml_diff>
--- a/requisitos-sistema/requisitos_estoque_cozinha.xlsx
+++ b/requisitos-sistema/requisitos_estoque_cozinha.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://institutogerminare-my.sharepoint.com/personal/davi_souza_institutojef_org_br/Documents/Área de Trabalho/GerminaT 2/inventra/engenharia-e-qualidade-de-software/requisitos-sistema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{61C9EADD-2906-4450-8165-81B34D94D9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66F54511-7A6D-46B5-A2FC-6BD16416E2F9}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{61C9EADD-2906-4450-8165-81B34D94D9E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8332AFA-69A1-4E35-83D6-9AF9B9685531}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="137">
   <si>
     <t>Código</t>
   </si>
@@ -326,21 +326,12 @@
     <t>RF24</t>
   </si>
   <si>
-    <t>Pedido de compra automático</t>
-  </si>
-  <si>
     <t>Gerar pedido de compra para fornecedores baseado em ponto de pedido (estoque mínimo) e consumo médio.</t>
   </si>
   <si>
     <t>RF25</t>
   </si>
   <si>
-    <t>Previsão de consumo</t>
-  </si>
-  <si>
-    <t>Sugerir quantidade a ser comprada com base em histórico de consumo sazonal e tendências.</t>
-  </si>
-  <si>
     <t>RF26</t>
   </si>
   <si>
@@ -350,18 +341,6 @@
     <t>Enviar alertas de vencimento, estoque baixo, auditoria pendente e movimentações suspeitas.</t>
   </si>
   <si>
-    <t>RF27</t>
-  </si>
-  <si>
-    <t>RF28</t>
-  </si>
-  <si>
-    <t>Fechamento de inventário periódico</t>
-  </si>
-  <si>
-    <t>RF29</t>
-  </si>
-  <si>
     <t>Gestão de fornecedores</t>
   </si>
   <si>
@@ -374,9 +353,6 @@
     <t>Obrigar ou permitir registrar motivo na saída (ex: consumo, perda, doação, devolução a fornecedor).</t>
   </si>
   <si>
-    <t>Estoque mínimo por cozinha/período</t>
-  </si>
-  <si>
     <t>Cada movimentação deve permitir rastrear qual usuário, data/hora, terminal/IP e motivo – com cadeia de auditoria imutável.</t>
   </si>
   <si>
@@ -416,12 +392,6 @@
     <t>Permitir exportar produtos, movimentações e inventários via CSV/Excel.</t>
   </si>
   <si>
-    <t>Permitir "congelar" o estoque para contagem por mês. (View)</t>
-  </si>
-  <si>
-    <t>Definir nível mínimo de estoque diferente para dias úteis, finais de semana ou eventos. (input)</t>
-  </si>
-  <si>
     <t>Alerta de produto vencido</t>
   </si>
   <si>
@@ -450,6 +420,18 @@
   </si>
   <si>
     <t>RNF17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requisição de compra </t>
+  </si>
+  <si>
+    <t>RF20</t>
+  </si>
+  <si>
+    <t>Revisão de pedidos</t>
+  </si>
+  <si>
+    <t>Revisar produtos e suas quantidades antes de fazer a requisição.</t>
   </si>
 </sst>
 </file>
@@ -576,8 +558,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C92AE2FF-755C-4500-BBA2-265A9C2A3D10}" name="Tabela1" displayName="Tabela1" ref="A1:C29" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:C29" xr:uid="{C92AE2FF-755C-4500-BBA2-265A9C2A3D10}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C92AE2FF-755C-4500-BBA2-265A9C2A3D10}" name="Tabela1" displayName="Tabela1" ref="A1:C27" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:C27" xr:uid="{C92AE2FF-755C-4500-BBA2-265A9C2A3D10}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{C7205364-51EA-4410-8A03-368DA3CA1DA5}" name="Código" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{F6C5F0B6-B179-41B7-BECF-69D1011F0C93}" name="Título"/>
@@ -884,7 +866,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
@@ -982,7 +964,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="B9" t="s">
         <v>28</v>
@@ -1004,7 +986,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B11" t="s">
         <v>34</v>
@@ -1112,111 +1094,89 @@
         <v>61</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>56</v>
+        <v>134</v>
       </c>
       <c r="B21" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21" t="s">
         <v>101</v>
-      </c>
-      <c r="C21" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B22" t="s">
-        <v>104</v>
+        <v>135</v>
       </c>
       <c r="C22" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="B23" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C23" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B24" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C24" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B25" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C25" t="s">
-        <v>131</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C26" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B27" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="C27" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="B28" t="s">
-        <v>117</v>
-      </c>
-      <c r="C28" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B29" t="s">
-        <v>133</v>
-      </c>
-      <c r="C29" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>135</v>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1377,7 +1337,7 @@
         <v>98</v>
       </c>
       <c r="C13" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1385,10 +1345,10 @@
         <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C14" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -1396,48 +1356,48 @@
         <v>97</v>
       </c>
       <c r="B15" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="C15" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="B16" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C16" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C17" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="B18" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" t="s">
         <v>127</v>
-      </c>
-      <c r="C18" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B19" t="s">
         <v>22</v>

</xml_diff>